<commit_message>
Guardado automatico, eliminar alumno, mapa con diseno anterior e impresion de reportes, fase final a probar
</commit_message>
<xml_diff>
--- a/PlanesEstudio/Plan_Economia_2024.xlsx
+++ b/PlanesEstudio/Plan_Economia_2024.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -440,6 +440,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -468,6 +469,11 @@
           <t>Prerrequisitos</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -487,6 +493,11 @@
         </is>
       </c>
       <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -506,6 +517,11 @@
         </is>
       </c>
       <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -525,6 +541,11 @@
         </is>
       </c>
       <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -544,6 +565,11 @@
         </is>
       </c>
       <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -563,6 +589,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -586,6 +613,11 @@
           <t>Lengua I</t>
         </is>
       </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -605,6 +637,11 @@
         </is>
       </c>
       <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -624,6 +661,11 @@
         </is>
       </c>
       <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -643,6 +685,11 @@
         </is>
       </c>
       <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -662,6 +709,11 @@
         </is>
       </c>
       <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -685,6 +737,11 @@
           <t>Cálculo I</t>
         </is>
       </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -708,6 +765,11 @@
           <t>Cálculo I</t>
         </is>
       </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -731,6 +793,11 @@
           <t>Cálculo I</t>
         </is>
       </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -750,6 +817,11 @@
         </is>
       </c>
       <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -769,6 +841,11 @@
         </is>
       </c>
       <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -788,6 +865,11 @@
         </is>
       </c>
       <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -811,6 +893,11 @@
           <t>Microeconomía II</t>
         </is>
       </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -830,6 +917,11 @@
         </is>
       </c>
       <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -849,6 +941,11 @@
         </is>
       </c>
       <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -868,6 +965,11 @@
         </is>
       </c>
       <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -887,6 +989,11 @@
         </is>
       </c>
       <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -906,6 +1013,11 @@
         </is>
       </c>
       <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -929,6 +1041,11 @@
           <t>Macroeconomía I</t>
         </is>
       </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -952,6 +1069,11 @@
           <t>Estadística</t>
         </is>
       </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -971,6 +1093,11 @@
         </is>
       </c>
       <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -994,6 +1121,11 @@
           <t>Economía mexicana I</t>
         </is>
       </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1013,6 +1145,11 @@
         </is>
       </c>
       <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1032,6 +1169,7 @@
         </is>
       </c>
       <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1055,6 +1193,11 @@
           <t>Microeconomía III, Organización industrial</t>
         </is>
       </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1078,6 +1221,11 @@
           <t>Macroeconomía II</t>
         </is>
       </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1101,6 +1249,11 @@
           <t>Econometría I</t>
         </is>
       </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -1124,6 +1277,11 @@
           <t>Econometría I</t>
         </is>
       </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1143,6 +1301,11 @@
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1162,6 +1325,11 @@
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -1181,6 +1349,7 @@
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -1200,6 +1369,11 @@
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -1219,6 +1393,11 @@
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -1238,6 +1417,11 @@
         </is>
       </c>
       <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -1257,6 +1441,11 @@
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -1276,6 +1465,7 @@
         </is>
       </c>
       <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -1295,6 +1485,11 @@
         </is>
       </c>
       <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -1314,6 +1509,11 @@
         </is>
       </c>
       <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -1333,6 +1533,11 @@
         </is>
       </c>
       <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Disciplinar</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -1352,6 +1557,11 @@
         </is>
       </c>
       <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -1371,6 +1581,7 @@
         </is>
       </c>
       <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -1390,6 +1601,7 @@
         </is>
       </c>
       <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -1409,6 +1621,7 @@
         </is>
       </c>
       <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Materias de varios periodos: servicio social dura hasta 2 y no se marca como rezago mientras sigue en curso
- Columna H de la plantilla: periodos que dura la materia (vacía = 1; servicio social = 2)
- Rezago, alertas, reportes y reporte del periodo toman como en curso la materia que sigue cursando
  desde un periodo anterior dentro de su duración; pasado ese plazo sin resultado sí es rezago
- Reporte del periodo: al cerrar el primer periodo aparece como "Continúa el siguiente periodo"
- Pantalla: aviso al abrirla en el periodo siguiente y se puede registrar ahí su resultado

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PlanesEstudio/Plan_Economia_2024.xlsx
+++ b/PlanesEstudio/Plan_Economia_2024.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.139196" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -487,6 +487,7 @@
     <col width="48" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -525,6 +526,11 @@
           <t>Creditos minimos (%)</t>
         </is>
       </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Periodos que dura</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -550,6 +556,7 @@
         </is>
       </c>
       <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -575,6 +582,7 @@
         </is>
       </c>
       <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -600,6 +608,7 @@
         </is>
       </c>
       <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -625,6 +634,7 @@
         </is>
       </c>
       <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -646,6 +656,7 @@
       <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -675,6 +686,7 @@
         </is>
       </c>
       <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -700,6 +712,7 @@
         </is>
       </c>
       <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -725,6 +738,7 @@
         </is>
       </c>
       <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -750,6 +764,7 @@
         </is>
       </c>
       <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -775,6 +790,7 @@
         </is>
       </c>
       <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -804,6 +820,7 @@
         </is>
       </c>
       <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -833,6 +850,7 @@
         </is>
       </c>
       <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -862,6 +880,7 @@
         </is>
       </c>
       <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -887,6 +906,7 @@
         </is>
       </c>
       <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -912,6 +932,7 @@
         </is>
       </c>
       <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -937,6 +958,7 @@
         </is>
       </c>
       <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -966,6 +988,7 @@
         </is>
       </c>
       <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -991,6 +1014,7 @@
         </is>
       </c>
       <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1016,6 +1040,7 @@
         </is>
       </c>
       <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1041,6 +1066,7 @@
         </is>
       </c>
       <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1066,6 +1092,7 @@
         </is>
       </c>
       <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1091,6 +1118,7 @@
         </is>
       </c>
       <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1120,6 +1148,7 @@
         </is>
       </c>
       <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1149,6 +1178,7 @@
         </is>
       </c>
       <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1174,6 +1204,7 @@
         </is>
       </c>
       <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1203,6 +1234,7 @@
         </is>
       </c>
       <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1228,6 +1260,7 @@
         </is>
       </c>
       <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1249,6 +1282,7 @@
       <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1278,6 +1312,7 @@
         </is>
       </c>
       <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1307,6 +1342,7 @@
         </is>
       </c>
       <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1336,6 +1372,7 @@
         </is>
       </c>
       <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -1365,6 +1402,7 @@
         </is>
       </c>
       <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1390,6 +1428,7 @@
         </is>
       </c>
       <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1415,6 +1454,7 @@
         </is>
       </c>
       <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -1436,6 +1476,7 @@
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -1461,6 +1502,7 @@
         </is>
       </c>
       <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -1486,6 +1528,7 @@
         </is>
       </c>
       <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -1511,6 +1554,7 @@
         </is>
       </c>
       <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -1538,6 +1582,9 @@
       <c r="G40" s="2" t="n">
         <v>70</v>
       </c>
+      <c r="H40" s="2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -1559,6 +1606,7 @@
       <c r="E41" s="2" t="n"/>
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -1586,6 +1634,7 @@
       <c r="G42" s="2" t="n">
         <v>70</v>
       </c>
+      <c r="H42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -1611,6 +1660,7 @@
         </is>
       </c>
       <c r="G43" s="2" t="n"/>
+      <c r="H43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -1636,6 +1686,7 @@
         </is>
       </c>
       <c r="G44" s="2" t="n"/>
+      <c r="H44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -1663,6 +1714,7 @@
       <c r="G45" s="2" t="n">
         <v>70</v>
       </c>
+      <c r="H45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n"/>
@@ -1682,6 +1734,7 @@
       <c r="E46" s="2" t="n"/>
       <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="n"/>
+      <c r="H46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
@@ -1701,6 +1754,7 @@
       <c r="E47" s="2" t="n"/>
       <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="n"/>
+      <c r="H47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n"/>
@@ -1720,6 +1774,7 @@
       <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="n"/>
+      <c r="H48" s="2" t="n"/>
     </row>
     <row r="49"/>
   </sheetData>

</xml_diff>

<commit_message>
Planes: áreas AFBG e Iniciación a la disciplina
Columna Area, lista desplegable e instrucciones de los planes con los nombres
oficiales de la UV.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PlanesEstudio/Plan_Economia_2024.xlsx
+++ b/PlanesEstudio/Plan_Economia_2024.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.139196" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -485,7 +485,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
@@ -552,7 +552,7 @@
       <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>AFBG</t>
         </is>
       </c>
       <c r="G2" s="2" t="n"/>
@@ -578,7 +578,7 @@
       <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>AFBG</t>
         </is>
       </c>
       <c r="G3" s="2" t="n"/>
@@ -604,7 +604,7 @@
       <c r="E4" s="2" t="n"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>AFBG</t>
         </is>
       </c>
       <c r="G4" s="2" t="n"/>
@@ -630,7 +630,7 @@
       <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>Iniciación a la disciplina</t>
         </is>
       </c>
       <c r="G5" s="2" t="n"/>
@@ -682,7 +682,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>AFBG</t>
         </is>
       </c>
       <c r="G7" s="2" t="n"/>
@@ -708,7 +708,7 @@
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>AFBG</t>
         </is>
       </c>
       <c r="G8" s="2" t="n"/>
@@ -734,7 +734,7 @@
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>Iniciación a la disciplina</t>
         </is>
       </c>
       <c r="G9" s="2" t="n"/>
@@ -760,7 +760,7 @@
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>Iniciación a la disciplina</t>
         </is>
       </c>
       <c r="G10" s="2" t="n"/>
@@ -786,7 +786,7 @@
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>Iniciación a la disciplina</t>
         </is>
       </c>
       <c r="G11" s="2" t="n"/>
@@ -902,7 +902,7 @@
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>Iniciación a la disciplina</t>
         </is>
       </c>
       <c r="G15" s="2" t="n"/>
@@ -928,7 +928,7 @@
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>Iniciación a la disciplina</t>
         </is>
       </c>
       <c r="G16" s="2" t="n"/>
@@ -954,7 +954,7 @@
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>AFBG</t>
         </is>
       </c>
       <c r="G17" s="2" t="n"/>
@@ -1088,7 +1088,7 @@
       <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>Iniciación a la disciplina</t>
         </is>
       </c>
       <c r="G22" s="2" t="n"/>
@@ -1776,7 +1776,6 @@
       <c r="G48" s="2" t="n"/>
       <c r="H48" s="2" t="n"/>
     </row>
-    <row r="49"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>